<commit_message>
More RoC, Wenyan scorer, Manyogana
I'm gonna sort out a periodization + wenyan scoring system to get everything in the corpus organised. Then, a metadata audit and display.

Wenyan scorer will see its own individual release once its efficacy has proven itself to me. Right now though it's doing pretty damn good.
</commit_message>
<xml_diff>
--- a/viewer/resources/wikipedia/manyogana_mora_table-wiki.xlsx
+++ b/viewer/resources/wikipedia/manyogana_mora_table-wiki.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7a415feeb18fead8/Documents/fanyahanwen-corpus/viewer/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7a415feeb18fead8/Documents/fanyahanwen-corpus/viewer/resources/wikipedia/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{67FC1C6F-5719-4AE1-86B4-DF1A9B64E965}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -1309,11 +1309,7 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="M6:M7"/>
-    <mergeCell ref="N6:N7"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="G8:G9"/>
-    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="J3:J4"/>
     <mergeCell ref="O8:O9"/>
     <mergeCell ref="K3:K4"/>
     <mergeCell ref="M3:M4"/>
@@ -1330,7 +1326,11 @@
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="F3:F4"/>
     <mergeCell ref="I3:I4"/>
-    <mergeCell ref="J3:J4"/>
+    <mergeCell ref="M6:M7"/>
+    <mergeCell ref="N6:N7"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="K8:K9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>